<commit_message>
Please provide the code changes or file diffs you would like me to summarize.
</commit_message>
<xml_diff>
--- a/HomeWork/Kỳ 2B/PHI501.22(Triết học)/Project/DSHV_Triết học kỳ SP26.xlsx
+++ b/HomeWork/Kỳ 2B/PHI501.22(Triết học)/Project/DSHV_Triết học kỳ SP26.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Đầu tư\Học Hành\IT\MSE\HomeWork\Kỳ 2B\PHI501.22(Triết học)\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7A9B3F-8247-48EA-A6AA-1D5535F93A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD48F353-9839-4613-BC26-B9B1954A9640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A1ECAD01-FCFA-4EDA-8010-939F0E30C442}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{A1ECAD01-FCFA-4EDA-8010-939F0E30C442}"/>
   </bookViews>
   <sheets>
     <sheet name="DS học Triết" sheetId="1" r:id="rId1"/>
@@ -420,7 +420,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="B1dd\-mmm\-yy"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -493,6 +493,19 @@
       <color theme="1"/>
       <name val="Open Sans"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -671,33 +684,6 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -710,21 +696,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -733,6 +704,48 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1070,39 +1083,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC2D7083-331B-45DA-9E86-8E36217E10C8}">
   <dimension ref="A1:G62"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="12" customWidth="1"/>
-    <col min="3" max="3" width="27.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" style="1" customWidth="1"/>
     <col min="4" max="4" width="11" style="4" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="50.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="50.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="8" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="35.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:7" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-    </row>
-    <row r="2" spans="1:7" ht="35.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="27" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+    </row>
+    <row r="2" spans="1:7" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>0</v>
       </c>
@@ -1123,11 +1136,11 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="16" t="s">
         <v>58</v>
       </c>
       <c r="C4" s="5" t="s">
@@ -1144,11 +1157,11 @@
       </c>
       <c r="G4" s="13"/>
     </row>
-    <row r="5" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="25"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="5" t="s">
         <v>23</v>
       </c>
@@ -1163,11 +1176,11 @@
       </c>
       <c r="G5" s="13"/>
     </row>
-    <row r="6" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>3</v>
       </c>
-      <c r="B6" s="25"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="5" t="s">
         <v>25</v>
       </c>
@@ -1182,11 +1195,11 @@
       </c>
       <c r="G6" s="13"/>
     </row>
-    <row r="7" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>4</v>
       </c>
-      <c r="B7" s="25"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="5" t="s">
         <v>26</v>
       </c>
@@ -1201,11 +1214,11 @@
       </c>
       <c r="G7" s="13"/>
     </row>
-    <row r="8" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>5</v>
       </c>
-      <c r="B8" s="25"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="5" t="s">
         <v>27</v>
       </c>
@@ -1220,11 +1233,11 @@
       </c>
       <c r="G8" s="13"/>
     </row>
-    <row r="9" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>6</v>
       </c>
-      <c r="B9" s="25"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="5" t="s">
         <v>29</v>
       </c>
@@ -1239,11 +1252,11 @@
       </c>
       <c r="G9" s="13"/>
     </row>
-    <row r="10" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>7</v>
       </c>
-      <c r="B10" s="25"/>
+      <c r="B10" s="16"/>
       <c r="C10" s="5" t="s">
         <v>31</v>
       </c>
@@ -1258,11 +1271,11 @@
       </c>
       <c r="G10" s="13"/>
     </row>
-    <row r="11" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>8</v>
       </c>
-      <c r="B11" s="25"/>
+      <c r="B11" s="16"/>
       <c r="C11" s="5" t="s">
         <v>32</v>
       </c>
@@ -1277,11 +1290,11 @@
       </c>
       <c r="G11" s="13"/>
     </row>
-    <row r="12" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>9</v>
       </c>
-      <c r="B12" s="25"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="5" t="s">
         <v>34</v>
       </c>
@@ -1296,11 +1309,11 @@
       </c>
       <c r="G12" s="13"/>
     </row>
-    <row r="13" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>10</v>
       </c>
-      <c r="B13" s="25"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="5" t="s">
         <v>35</v>
       </c>
@@ -1315,11 +1328,11 @@
       </c>
       <c r="G13" s="13"/>
     </row>
-    <row r="14" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>11</v>
       </c>
-      <c r="B14" s="25"/>
+      <c r="B14" s="16"/>
       <c r="C14" s="5" t="s">
         <v>37</v>
       </c>
@@ -1334,11 +1347,11 @@
       </c>
       <c r="G14" s="13"/>
     </row>
-    <row r="15" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>12</v>
       </c>
-      <c r="B15" s="25"/>
+      <c r="B15" s="16"/>
       <c r="C15" s="5" t="s">
         <v>39</v>
       </c>
@@ -1353,11 +1366,11 @@
       </c>
       <c r="G15" s="13"/>
     </row>
-    <row r="16" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>13</v>
       </c>
-      <c r="B16" s="25"/>
+      <c r="B16" s="16"/>
       <c r="C16" s="5" t="s">
         <v>41</v>
       </c>
@@ -1372,11 +1385,11 @@
       </c>
       <c r="G16" s="13"/>
     </row>
-    <row r="17" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>14</v>
       </c>
-      <c r="B17" s="25"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="5" t="s">
         <v>43</v>
       </c>
@@ -1391,11 +1404,11 @@
       </c>
       <c r="G17" s="13"/>
     </row>
-    <row r="18" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>15</v>
       </c>
-      <c r="B18" s="25"/>
+      <c r="B18" s="16"/>
       <c r="C18" s="5" t="s">
         <v>45</v>
       </c>
@@ -1410,11 +1423,11 @@
       </c>
       <c r="G18" s="13"/>
     </row>
-    <row r="19" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>16</v>
       </c>
-      <c r="B19" s="25"/>
+      <c r="B19" s="16"/>
       <c r="C19" s="5" t="s">
         <v>46</v>
       </c>
@@ -1429,11 +1442,11 @@
       </c>
       <c r="G19" s="13"/>
     </row>
-    <row r="20" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>17</v>
       </c>
-      <c r="B20" s="25"/>
+      <c r="B20" s="16"/>
       <c r="C20" s="5" t="s">
         <v>47</v>
       </c>
@@ -1448,11 +1461,11 @@
       </c>
       <c r="G20" s="13"/>
     </row>
-    <row r="21" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>18</v>
       </c>
-      <c r="B21" s="25"/>
+      <c r="B21" s="16"/>
       <c r="C21" s="5" t="s">
         <v>48</v>
       </c>
@@ -1467,11 +1480,11 @@
       </c>
       <c r="G21" s="13"/>
     </row>
-    <row r="22" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>19</v>
       </c>
-      <c r="B22" s="25"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="5" t="s">
         <v>50</v>
       </c>
@@ -1486,11 +1499,11 @@
       </c>
       <c r="G22" s="13"/>
     </row>
-    <row r="23" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>20</v>
       </c>
-      <c r="B23" s="25"/>
+      <c r="B23" s="16"/>
       <c r="C23" s="5" t="s">
         <v>52</v>
       </c>
@@ -1505,11 +1518,11 @@
       </c>
       <c r="G23" s="13"/>
     </row>
-    <row r="24" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>21</v>
       </c>
-      <c r="B24" s="25"/>
+      <c r="B24" s="16"/>
       <c r="C24" s="5" t="s">
         <v>54</v>
       </c>
@@ -1524,11 +1537,11 @@
       </c>
       <c r="G24" s="13"/>
     </row>
-    <row r="25" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>22</v>
       </c>
-      <c r="B25" s="25"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="5" t="s">
         <v>55</v>
       </c>
@@ -1543,11 +1556,11 @@
       </c>
       <c r="G25" s="13"/>
     </row>
-    <row r="26" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>23</v>
       </c>
-      <c r="B26" s="25"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="5" t="s">
         <v>56</v>
       </c>
@@ -1562,11 +1575,11 @@
       </c>
       <c r="G26" s="13"/>
     </row>
-    <row r="27" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>24</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="17" t="s">
         <v>65</v>
       </c>
       <c r="C27" s="5" t="s">
@@ -1583,11 +1596,11 @@
       </c>
       <c r="G27" s="13"/>
     </row>
-    <row r="28" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>25</v>
       </c>
-      <c r="B28" s="26"/>
+      <c r="B28" s="17"/>
       <c r="C28" s="5" t="s">
         <v>60</v>
       </c>
@@ -1602,11 +1615,11 @@
       </c>
       <c r="G28" s="13"/>
     </row>
-    <row r="29" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>26</v>
       </c>
-      <c r="B29" s="26"/>
+      <c r="B29" s="17"/>
       <c r="C29" s="5" t="s">
         <v>62</v>
       </c>
@@ -1621,11 +1634,11 @@
       </c>
       <c r="G29" s="13"/>
     </row>
-    <row r="30" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>27</v>
       </c>
-      <c r="B30" s="26"/>
+      <c r="B30" s="17"/>
       <c r="C30" s="5" t="s">
         <v>63</v>
       </c>
@@ -1640,11 +1653,11 @@
       </c>
       <c r="G30" s="13"/>
     </row>
-    <row r="31" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>28</v>
       </c>
-      <c r="B31" s="26" t="s">
+      <c r="B31" s="17" t="s">
         <v>66</v>
       </c>
       <c r="C31" s="5" t="s">
@@ -1661,11 +1674,11 @@
       </c>
       <c r="G31" s="13"/>
     </row>
-    <row r="32" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>29</v>
       </c>
-      <c r="B32" s="26"/>
+      <c r="B32" s="17"/>
       <c r="C32" s="5" t="s">
         <v>69</v>
       </c>
@@ -1680,11 +1693,11 @@
       </c>
       <c r="G32" s="13"/>
     </row>
-    <row r="33" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>30</v>
       </c>
-      <c r="B33" s="26"/>
+      <c r="B33" s="17"/>
       <c r="C33" s="5" t="s">
         <v>71</v>
       </c>
@@ -1699,11 +1712,11 @@
       </c>
       <c r="G33" s="13"/>
     </row>
-    <row r="34" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>31</v>
       </c>
-      <c r="B34" s="26"/>
+      <c r="B34" s="17"/>
       <c r="C34" s="5" t="s">
         <v>73</v>
       </c>
@@ -1718,11 +1731,11 @@
       </c>
       <c r="G34" s="13"/>
     </row>
-    <row r="35" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>32</v>
       </c>
-      <c r="B35" s="26"/>
+      <c r="B35" s="17"/>
       <c r="C35" s="5" t="s">
         <v>75</v>
       </c>
@@ -1737,11 +1750,11 @@
       </c>
       <c r="G35" s="13"/>
     </row>
-    <row r="36" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>33</v>
       </c>
-      <c r="B36" s="26"/>
+      <c r="B36" s="17"/>
       <c r="C36" s="5" t="s">
         <v>77</v>
       </c>
@@ -1756,11 +1769,11 @@
       </c>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>34</v>
       </c>
-      <c r="B37" s="26"/>
+      <c r="B37" s="17"/>
       <c r="C37" s="5" t="s">
         <v>78</v>
       </c>
@@ -1775,11 +1788,11 @@
       </c>
       <c r="G37" s="13"/>
     </row>
-    <row r="38" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>35</v>
       </c>
-      <c r="B38" s="26"/>
+      <c r="B38" s="17"/>
       <c r="C38" s="5" t="s">
         <v>80</v>
       </c>
@@ -1794,11 +1807,11 @@
       </c>
       <c r="G38" s="13"/>
     </row>
-    <row r="39" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>36</v>
       </c>
-      <c r="B39" s="26"/>
+      <c r="B39" s="17"/>
       <c r="C39" s="5" t="s">
         <v>82</v>
       </c>
@@ -1813,11 +1826,11 @@
       </c>
       <c r="G39" s="13"/>
     </row>
-    <row r="40" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
         <v>37</v>
       </c>
-      <c r="B40" s="26"/>
+      <c r="B40" s="17"/>
       <c r="C40" s="5" t="s">
         <v>84</v>
       </c>
@@ -1832,11 +1845,11 @@
       </c>
       <c r="G40" s="13"/>
     </row>
-    <row r="41" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>38</v>
       </c>
-      <c r="B41" s="26"/>
+      <c r="B41" s="17"/>
       <c r="C41" s="5" t="s">
         <v>86</v>
       </c>
@@ -1851,11 +1864,11 @@
       </c>
       <c r="G41" s="13"/>
     </row>
-    <row r="42" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>39</v>
       </c>
-      <c r="B42" s="26"/>
+      <c r="B42" s="17"/>
       <c r="C42" s="5" t="s">
         <v>88</v>
       </c>
@@ -1870,11 +1883,11 @@
       </c>
       <c r="G42" s="13"/>
     </row>
-    <row r="43" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>40</v>
       </c>
-      <c r="B43" s="26"/>
+      <c r="B43" s="17"/>
       <c r="C43" s="5" t="s">
         <v>90</v>
       </c>
@@ -1889,11 +1902,11 @@
       </c>
       <c r="G43" s="13"/>
     </row>
-    <row r="44" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
         <v>41</v>
       </c>
-      <c r="B44" s="26"/>
+      <c r="B44" s="17"/>
       <c r="C44" s="5" t="s">
         <v>92</v>
       </c>
@@ -1908,11 +1921,11 @@
       </c>
       <c r="G44" s="13"/>
     </row>
-    <row r="45" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="3">
         <v>42</v>
       </c>
-      <c r="B45" s="26"/>
+      <c r="B45" s="17"/>
       <c r="C45" s="5" t="s">
         <v>94</v>
       </c>
@@ -1927,11 +1940,11 @@
       </c>
       <c r="G45" s="13"/>
     </row>
-    <row r="46" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="3">
         <v>43</v>
       </c>
-      <c r="B46" s="26"/>
+      <c r="B46" s="17"/>
       <c r="C46" s="5" t="s">
         <v>96</v>
       </c>
@@ -1946,11 +1959,11 @@
       </c>
       <c r="G46" s="13"/>
     </row>
-    <row r="47" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
         <v>44</v>
       </c>
-      <c r="B47" s="26"/>
+      <c r="B47" s="17"/>
       <c r="C47" s="5" t="s">
         <v>98</v>
       </c>
@@ -1965,11 +1978,11 @@
       </c>
       <c r="G47" s="13"/>
     </row>
-    <row r="48" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="3">
         <v>45</v>
       </c>
-      <c r="B48" s="26"/>
+      <c r="B48" s="17"/>
       <c r="C48" s="5" t="s">
         <v>100</v>
       </c>
@@ -1984,11 +1997,11 @@
       </c>
       <c r="G48" s="13"/>
     </row>
-    <row r="49" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3">
         <v>46</v>
       </c>
-      <c r="B49" s="26"/>
+      <c r="B49" s="17"/>
       <c r="C49" s="5" t="s">
         <v>101</v>
       </c>
@@ -2003,11 +2016,11 @@
       </c>
       <c r="G49" s="13"/>
     </row>
-    <row r="50" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="3">
         <v>47</v>
       </c>
-      <c r="B50" s="26" t="s">
+      <c r="B50" s="17" t="s">
         <v>123</v>
       </c>
       <c r="C50" s="5" t="s">
@@ -2024,11 +2037,11 @@
       </c>
       <c r="G50" s="13"/>
     </row>
-    <row r="51" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="3">
         <v>48</v>
       </c>
-      <c r="B51" s="26"/>
+      <c r="B51" s="17"/>
       <c r="C51" s="5" t="s">
         <v>104</v>
       </c>
@@ -2043,11 +2056,11 @@
       </c>
       <c r="G51" s="13"/>
     </row>
-    <row r="52" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="3">
         <v>49</v>
       </c>
-      <c r="B52" s="26"/>
+      <c r="B52" s="17"/>
       <c r="C52" s="5" t="s">
         <v>106</v>
       </c>
@@ -2062,11 +2075,11 @@
       </c>
       <c r="G52" s="13"/>
     </row>
-    <row r="53" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="3">
         <v>50</v>
       </c>
-      <c r="B53" s="26"/>
+      <c r="B53" s="17"/>
       <c r="C53" s="5" t="s">
         <v>108</v>
       </c>
@@ -2081,11 +2094,11 @@
       </c>
       <c r="G53" s="13"/>
     </row>
-    <row r="54" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="3">
         <v>51</v>
       </c>
-      <c r="B54" s="26"/>
+      <c r="B54" s="17"/>
       <c r="C54" s="5" t="s">
         <v>109</v>
       </c>
@@ -2100,11 +2113,11 @@
       </c>
       <c r="G54" s="13"/>
     </row>
-    <row r="55" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="3">
         <v>52</v>
       </c>
-      <c r="B55" s="26"/>
+      <c r="B55" s="17"/>
       <c r="C55" s="5" t="s">
         <v>111</v>
       </c>
@@ -2119,11 +2132,11 @@
       </c>
       <c r="G55" s="13"/>
     </row>
-    <row r="56" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="3">
         <v>53</v>
       </c>
-      <c r="B56" s="26"/>
+      <c r="B56" s="17"/>
       <c r="C56" s="5" t="s">
         <v>113</v>
       </c>
@@ -2138,11 +2151,11 @@
       </c>
       <c r="G56" s="13"/>
     </row>
-    <row r="57" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="3">
         <v>54</v>
       </c>
-      <c r="B57" s="26"/>
+      <c r="B57" s="17"/>
       <c r="C57" s="5" t="s">
         <v>115</v>
       </c>
@@ -2157,11 +2170,11 @@
       </c>
       <c r="G57" s="13"/>
     </row>
-    <row r="58" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="3">
         <v>55</v>
       </c>
-      <c r="B58" s="26"/>
+      <c r="B58" s="17"/>
       <c r="C58" s="5" t="s">
         <v>117</v>
       </c>
@@ -2176,11 +2189,11 @@
       </c>
       <c r="G58" s="13"/>
     </row>
-    <row r="59" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="3">
         <v>56</v>
       </c>
-      <c r="B59" s="26"/>
+      <c r="B59" s="17"/>
       <c r="C59" s="5" t="s">
         <v>119</v>
       </c>
@@ -2195,11 +2208,11 @@
       </c>
       <c r="G59" s="13"/>
     </row>
-    <row r="60" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="3">
         <v>57</v>
       </c>
-      <c r="B60" s="26"/>
+      <c r="B60" s="17"/>
       <c r="C60" s="5" t="s">
         <v>121</v>
       </c>
@@ -2214,7 +2227,7 @@
       </c>
       <c r="G60" s="13"/>
     </row>
-    <row r="61" spans="1:7" ht="102" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" ht="102" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="3">
         <v>58</v>
       </c>
@@ -2235,26 +2248,26 @@
       </c>
       <c r="G61" s="13"/>
     </row>
-    <row r="62" spans="1:7" ht="25.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="33" t="s">
+    <row r="62" spans="1:7" ht="25.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="B62" s="34"/>
-      <c r="C62" s="34"/>
-      <c r="D62" s="34"/>
-      <c r="E62" s="34"/>
-      <c r="F62" s="34"/>
-      <c r="G62" s="35"/>
+      <c r="B62" s="20"/>
+      <c r="C62" s="20"/>
+      <c r="D62" s="20"/>
+      <c r="E62" s="20"/>
+      <c r="F62" s="20"/>
+      <c r="G62" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A62:G62"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B4:B26"/>
     <mergeCell ref="B27:B30"/>
     <mergeCell ref="B31:B49"/>
     <mergeCell ref="B50:B60"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A62:G62"/>
   </mergeCells>
   <conditionalFormatting sqref="C1 C3:C61 C63:C1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="5"/>
@@ -2271,1099 +2284,1100 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A929CC-90D6-433F-8CF3-61B220B19D5E}">
   <dimension ref="A1:F60"/>
-  <sheetFormatPr defaultColWidth="20" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="20" defaultRowHeight="18" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" style="15" customWidth="1"/>
-    <col min="2" max="2" width="10.77734375" style="20" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" style="18" customWidth="1"/>
-    <col min="4" max="4" width="28.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.77734375" style="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="20" style="15"/>
+    <col min="1" max="1" width="7.7109375" style="22" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" style="23" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" style="24" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" style="24" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.28515625" style="24" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" style="22" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="20" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:6" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-    </row>
-    <row r="2" spans="1:6" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="26"/>
+    </row>
+    <row r="2" spans="1:6" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="27" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="17">
+    <row r="3" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="28">
         <v>1</v>
       </c>
-      <c r="B3" s="28">
+      <c r="B3" s="29">
         <v>1</v>
       </c>
-      <c r="C3" s="17">
+      <c r="C3" s="28">
         <v>1</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="22">
+      <c r="E3" s="30">
         <v>35779</v>
       </c>
-      <c r="F3" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="17">
+      <c r="F3" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="28">
         <v>2</v>
       </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="17">
+      <c r="B4" s="29"/>
+      <c r="C4" s="28">
         <v>2</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="22">
+      <c r="E4" s="30">
         <v>36304</v>
       </c>
-      <c r="F4" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="17">
-        <v>3</v>
-      </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="17">
-        <v>3</v>
-      </c>
-      <c r="D5" s="21" t="s">
+      <c r="F4" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="28">
+        <v>3</v>
+      </c>
+      <c r="B5" s="29"/>
+      <c r="C5" s="28">
+        <v>3</v>
+      </c>
+      <c r="D5" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="30">
         <v>36708</v>
       </c>
-      <c r="F5" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="17">
-        <v>4</v>
-      </c>
-      <c r="B6" s="28"/>
-      <c r="C6" s="17">
-        <v>4</v>
-      </c>
-      <c r="D6" s="21" t="s">
+      <c r="F5" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="28">
+        <v>4</v>
+      </c>
+      <c r="B6" s="29"/>
+      <c r="C6" s="28">
+        <v>4</v>
+      </c>
+      <c r="D6" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="30">
         <v>35504</v>
       </c>
-      <c r="F6" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="17">
+      <c r="F6" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="28">
         <v>5</v>
       </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="17">
+      <c r="B7" s="29"/>
+      <c r="C7" s="28">
         <v>5</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="30">
         <v>36344</v>
       </c>
-      <c r="F7" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="17">
+      <c r="F7" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="28">
         <v>6</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="17">
+      <c r="B8" s="29"/>
+      <c r="C8" s="28">
         <v>6</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="30">
         <v>36505</v>
       </c>
-      <c r="F8" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="17">
+      <c r="F8" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="28">
         <v>7</v>
       </c>
-      <c r="B9" s="28"/>
-      <c r="C9" s="17">
+      <c r="B9" s="29"/>
+      <c r="C9" s="28">
         <v>7</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="30">
         <v>37114</v>
       </c>
-      <c r="F9" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="17">
+      <c r="F9" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="28">
         <v>8</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="17">
+      <c r="B10" s="29"/>
+      <c r="C10" s="28">
         <v>8</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="30">
         <v>34966</v>
       </c>
-      <c r="F10" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="17">
+      <c r="F10" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="28">
         <v>9</v>
       </c>
-      <c r="B11" s="28"/>
-      <c r="C11" s="17">
+      <c r="B11" s="29"/>
+      <c r="C11" s="28">
         <v>9</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="D11" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="30">
         <v>36969</v>
       </c>
-      <c r="F11" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17">
+      <c r="F11" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="28">
         <v>10</v>
       </c>
-      <c r="B12" s="28"/>
-      <c r="C12" s="17">
+      <c r="B12" s="29"/>
+      <c r="C12" s="28">
         <v>10</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="30">
         <v>36885</v>
       </c>
-      <c r="F12" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="17">
+      <c r="F12" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="28">
         <v>11</v>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="29">
         <v>2</v>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="28">
         <v>1</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="D13" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="30">
         <v>37497</v>
       </c>
-      <c r="F13" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="17">
+      <c r="F13" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="28">
         <v>12</v>
       </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="17">
+      <c r="B14" s="29"/>
+      <c r="C14" s="28">
         <v>2</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="30">
         <v>35912</v>
       </c>
-      <c r="F14" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="17">
+      <c r="F14" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="28">
         <v>13</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="17">
-        <v>3</v>
-      </c>
-      <c r="D15" s="21" t="s">
+      <c r="B15" s="29"/>
+      <c r="C15" s="28">
+        <v>3</v>
+      </c>
+      <c r="D15" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="30">
         <v>36755</v>
       </c>
-      <c r="F15" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="17">
+      <c r="F15" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="28">
         <v>14</v>
       </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="17">
-        <v>4</v>
-      </c>
-      <c r="D16" s="21" t="s">
+      <c r="B16" s="29"/>
+      <c r="C16" s="28">
+        <v>4</v>
+      </c>
+      <c r="D16" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="30">
         <v>31975</v>
       </c>
-      <c r="F16" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="17">
+      <c r="F16" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="28">
         <v>15</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="17">
+      <c r="B17" s="29"/>
+      <c r="C17" s="28">
         <v>5</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="D17" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="30">
         <v>36489</v>
       </c>
-      <c r="F17" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="17">
+      <c r="F17" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="28">
         <v>16</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="17">
+      <c r="B18" s="29"/>
+      <c r="C18" s="28">
         <v>6</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="D18" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="30">
         <v>34253</v>
       </c>
-      <c r="F18" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="17">
+      <c r="F18" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="28">
         <v>17</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="17">
+      <c r="B19" s="29"/>
+      <c r="C19" s="28">
         <v>7</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="D19" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="E19" s="22">
+      <c r="E19" s="30">
         <v>34866</v>
       </c>
-      <c r="F19" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="17">
+      <c r="F19" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="28">
         <v>18</v>
       </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="17">
+      <c r="B20" s="29"/>
+      <c r="C20" s="28">
         <v>8</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="30">
         <v>35242</v>
       </c>
-      <c r="F20" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="17">
+      <c r="F20" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="28">
         <v>19</v>
       </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="17">
+      <c r="B21" s="29"/>
+      <c r="C21" s="28">
         <v>9</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="D21" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="E21" s="22">
+      <c r="E21" s="30">
         <v>36810</v>
       </c>
-      <c r="F21" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="17">
+      <c r="F21" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="28">
         <v>20</v>
       </c>
-      <c r="B22" s="28">
-        <v>3</v>
-      </c>
-      <c r="C22" s="17">
+      <c r="B22" s="29">
+        <v>3</v>
+      </c>
+      <c r="C22" s="28">
         <v>1</v>
       </c>
-      <c r="D22" s="21" t="s">
+      <c r="D22" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="E22" s="22">
+      <c r="E22" s="30">
         <v>34999</v>
       </c>
-      <c r="F22" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="17">
+      <c r="F22" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="28">
         <v>21</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="17">
+      <c r="B23" s="29"/>
+      <c r="C23" s="28">
         <v>2</v>
       </c>
-      <c r="D23" s="21" t="s">
+      <c r="D23" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="22">
+      <c r="E23" s="30">
         <v>36105</v>
       </c>
-      <c r="F23" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="17">
+      <c r="F23" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="28">
         <v>22</v>
       </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="17">
-        <v>3</v>
-      </c>
-      <c r="D24" s="21" t="s">
+      <c r="B24" s="29"/>
+      <c r="C24" s="28">
+        <v>3</v>
+      </c>
+      <c r="D24" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="E24" s="22">
+      <c r="E24" s="30">
         <v>35935</v>
       </c>
-      <c r="F24" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="17">
+      <c r="F24" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="28">
         <v>23</v>
       </c>
-      <c r="B25" s="28"/>
-      <c r="C25" s="17">
-        <v>4</v>
-      </c>
-      <c r="D25" s="21" t="s">
+      <c r="B25" s="29"/>
+      <c r="C25" s="28">
+        <v>4</v>
+      </c>
+      <c r="D25" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="22">
+      <c r="E25" s="30">
         <v>36153</v>
       </c>
-      <c r="F25" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="17">
+      <c r="F25" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="28">
         <v>24</v>
       </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="17">
+      <c r="B26" s="29"/>
+      <c r="C26" s="28">
         <v>5</v>
       </c>
-      <c r="D26" s="21" t="s">
+      <c r="D26" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="E26" s="22">
+      <c r="E26" s="30">
         <v>35767</v>
       </c>
-      <c r="F26" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="17">
+      <c r="F26" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="28">
         <v>25</v>
       </c>
-      <c r="B27" s="28"/>
-      <c r="C27" s="17">
+      <c r="B27" s="29"/>
+      <c r="C27" s="28">
         <v>6</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="D27" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="E27" s="22">
+      <c r="E27" s="30">
         <v>30011</v>
       </c>
-      <c r="F27" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="17">
+      <c r="F27" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="28">
         <v>26</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="17">
+      <c r="B28" s="29"/>
+      <c r="C28" s="28">
         <v>7</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="D28" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="E28" s="22">
+      <c r="E28" s="30">
         <v>33890</v>
       </c>
-      <c r="F28" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="17">
+      <c r="F28" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="28">
         <v>27</v>
       </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="17">
+      <c r="B29" s="29"/>
+      <c r="C29" s="28">
         <v>8</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="E29" s="22">
+      <c r="E29" s="30">
         <v>32716</v>
       </c>
-      <c r="F29" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="17">
+      <c r="F29" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="28">
         <v>28</v>
       </c>
-      <c r="B30" s="28">
-        <v>4</v>
-      </c>
-      <c r="C30" s="17">
+      <c r="B30" s="29">
+        <v>4</v>
+      </c>
+      <c r="C30" s="28">
         <v>1</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="D30" s="28" t="s">
         <v>73</v>
       </c>
-      <c r="E30" s="22">
+      <c r="E30" s="30">
         <v>36976</v>
       </c>
-      <c r="F30" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="17">
+      <c r="F30" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="28">
         <v>29</v>
       </c>
-      <c r="B31" s="28"/>
-      <c r="C31" s="17">
+      <c r="B31" s="29"/>
+      <c r="C31" s="28">
         <v>2</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="E31" s="22">
+      <c r="E31" s="30">
         <v>30686</v>
       </c>
-      <c r="F31" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="17">
+      <c r="F31" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="28">
         <v>30</v>
       </c>
-      <c r="B32" s="28"/>
-      <c r="C32" s="17">
-        <v>3</v>
-      </c>
-      <c r="D32" s="21" t="s">
+      <c r="B32" s="29"/>
+      <c r="C32" s="28">
+        <v>3</v>
+      </c>
+      <c r="D32" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="E32" s="22">
+      <c r="E32" s="30">
         <v>32353</v>
       </c>
-      <c r="F32" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="17">
+      <c r="F32" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="28">
         <v>31</v>
       </c>
-      <c r="B33" s="28"/>
-      <c r="C33" s="17">
-        <v>4</v>
-      </c>
-      <c r="D33" s="21" t="s">
+      <c r="B33" s="29"/>
+      <c r="C33" s="28">
+        <v>4</v>
+      </c>
+      <c r="D33" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="E33" s="22">
+      <c r="E33" s="30">
         <v>36195</v>
       </c>
-      <c r="F33" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="17">
+      <c r="F33" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="28">
         <v>32</v>
       </c>
-      <c r="B34" s="28"/>
-      <c r="C34" s="17">
+      <c r="B34" s="29"/>
+      <c r="C34" s="28">
         <v>5</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="D34" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="E34" s="22">
+      <c r="E34" s="30">
         <v>37554</v>
       </c>
-      <c r="F34" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="17">
+      <c r="F34" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="28">
         <v>33</v>
       </c>
-      <c r="B35" s="28"/>
-      <c r="C35" s="17">
+      <c r="B35" s="29"/>
+      <c r="C35" s="28">
         <v>6</v>
       </c>
-      <c r="D35" s="21" t="s">
+      <c r="D35" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="E35" s="22">
+      <c r="E35" s="30">
         <v>35023</v>
       </c>
-      <c r="F35" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="17">
+      <c r="F35" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="28">
         <v>34</v>
       </c>
-      <c r="B36" s="28"/>
-      <c r="C36" s="17">
+      <c r="B36" s="29"/>
+      <c r="C36" s="28">
         <v>7</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="D36" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="E36" s="22">
+      <c r="E36" s="30">
         <v>32264</v>
       </c>
-      <c r="F36" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="17">
+      <c r="F36" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="28">
         <v>35</v>
       </c>
-      <c r="B37" s="28"/>
-      <c r="C37" s="17">
+      <c r="B37" s="29"/>
+      <c r="C37" s="28">
         <v>8</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="D37" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="22">
+      <c r="E37" s="30">
         <v>30945</v>
       </c>
-      <c r="F37" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="17">
+      <c r="F37" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="28">
         <v>36</v>
       </c>
-      <c r="B38" s="28"/>
-      <c r="C38" s="17">
+      <c r="B38" s="29"/>
+      <c r="C38" s="28">
         <v>9</v>
       </c>
-      <c r="D38" s="21" t="s">
+      <c r="D38" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="E38" s="22">
+      <c r="E38" s="30">
         <v>32348</v>
       </c>
-      <c r="F38" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="17">
+      <c r="F38" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="28">
         <v>37</v>
       </c>
-      <c r="B39" s="28"/>
-      <c r="C39" s="17">
+      <c r="B39" s="29"/>
+      <c r="C39" s="28">
         <v>10</v>
       </c>
-      <c r="D39" s="21" t="s">
+      <c r="D39" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="E39" s="22">
+      <c r="E39" s="30">
         <v>29907</v>
       </c>
-      <c r="F39" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="17">
+      <c r="F39" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="28">
         <v>38</v>
       </c>
-      <c r="B40" s="28">
+      <c r="B40" s="29">
         <v>5</v>
       </c>
-      <c r="C40" s="17">
+      <c r="C40" s="28">
         <v>1</v>
       </c>
-      <c r="D40" s="21" t="s">
+      <c r="D40" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="E40" s="22">
+      <c r="E40" s="30">
         <v>30213</v>
       </c>
-      <c r="F40" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="17">
+      <c r="F40" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="28">
         <v>39</v>
       </c>
-      <c r="B41" s="28"/>
-      <c r="C41" s="17">
+      <c r="B41" s="29"/>
+      <c r="C41" s="28">
         <v>2</v>
       </c>
-      <c r="D41" s="21" t="s">
+      <c r="D41" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="E41" s="22">
+      <c r="E41" s="30">
         <v>37753</v>
       </c>
-      <c r="F41" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="17">
+      <c r="F41" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="28">
         <v>40</v>
       </c>
-      <c r="B42" s="28"/>
-      <c r="C42" s="17">
-        <v>3</v>
-      </c>
-      <c r="D42" s="21" t="s">
+      <c r="B42" s="29"/>
+      <c r="C42" s="28">
+        <v>3</v>
+      </c>
+      <c r="D42" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="E42" s="22">
+      <c r="E42" s="30">
         <v>34201</v>
       </c>
-      <c r="F42" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="17">
+      <c r="F42" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="28">
         <v>41</v>
       </c>
-      <c r="B43" s="28"/>
-      <c r="C43" s="17">
-        <v>4</v>
-      </c>
-      <c r="D43" s="21" t="s">
+      <c r="B43" s="29"/>
+      <c r="C43" s="28">
+        <v>4</v>
+      </c>
+      <c r="D43" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="E43" s="22">
+      <c r="E43" s="30">
         <v>32633</v>
       </c>
-      <c r="F43" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="17">
+      <c r="F43" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="28">
         <v>42</v>
       </c>
-      <c r="B44" s="28"/>
-      <c r="C44" s="17">
+      <c r="B44" s="29"/>
+      <c r="C44" s="28">
         <v>5</v>
       </c>
-      <c r="D44" s="21" t="s">
+      <c r="D44" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="E44" s="22">
+      <c r="E44" s="30">
         <v>30251</v>
       </c>
-      <c r="F44" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="17">
+      <c r="F44" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="28">
         <v>43</v>
       </c>
-      <c r="B45" s="28"/>
-      <c r="C45" s="17">
+      <c r="B45" s="29"/>
+      <c r="C45" s="28">
         <v>6</v>
       </c>
-      <c r="D45" s="21" t="s">
+      <c r="D45" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="E45" s="22">
+      <c r="E45" s="30">
         <v>37868</v>
       </c>
-      <c r="F45" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="17">
+      <c r="F45" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="28">
         <v>44</v>
       </c>
-      <c r="B46" s="28"/>
-      <c r="C46" s="17">
+      <c r="B46" s="29"/>
+      <c r="C46" s="28">
         <v>7</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="D46" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="E46" s="22">
+      <c r="E46" s="30">
         <v>33022</v>
       </c>
-      <c r="F46" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="17">
+      <c r="F46" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="28">
         <v>45</v>
       </c>
-      <c r="B47" s="28"/>
-      <c r="C47" s="17">
+      <c r="B47" s="29"/>
+      <c r="C47" s="28">
         <v>8</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="D47" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="E47" s="22">
+      <c r="E47" s="30">
         <v>37548</v>
       </c>
-      <c r="F47" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="17">
+      <c r="F47" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="28">
         <v>46</v>
       </c>
-      <c r="B48" s="28"/>
-      <c r="C48" s="17">
+      <c r="B48" s="29"/>
+      <c r="C48" s="28">
         <v>9</v>
       </c>
-      <c r="D48" s="21" t="s">
+      <c r="D48" s="28" t="s">
         <v>71</v>
       </c>
-      <c r="E48" s="22">
+      <c r="E48" s="30">
         <v>37383</v>
       </c>
-      <c r="F48" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="17">
+      <c r="F48" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="28">
         <v>47</v>
       </c>
-      <c r="B49" s="28"/>
-      <c r="C49" s="17">
+      <c r="B49" s="29"/>
+      <c r="C49" s="28">
         <v>10</v>
       </c>
-      <c r="D49" s="19" t="s">
+      <c r="D49" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E49" s="35">
         <v>35114</v>
       </c>
-      <c r="F49" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="17">
+      <c r="F49" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="28">
         <v>48</v>
       </c>
-      <c r="B50" s="30">
+      <c r="B50" s="32">
         <v>6</v>
       </c>
-      <c r="C50" s="17">
+      <c r="C50" s="28">
         <v>1</v>
       </c>
-      <c r="D50" s="21" t="s">
+      <c r="D50" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="E50" s="10">
+      <c r="E50" s="30">
         <v>32628</v>
       </c>
-      <c r="F50" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" s="18" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="17">
+      <c r="F50" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" s="24" customFormat="1" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="28">
         <v>49</v>
       </c>
-      <c r="B51" s="31"/>
-      <c r="C51" s="17">
+      <c r="B51" s="33"/>
+      <c r="C51" s="28">
         <v>2</v>
       </c>
-      <c r="D51" s="21" t="s">
+      <c r="D51" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="E51" s="22">
+      <c r="E51" s="30">
         <v>37594</v>
       </c>
-      <c r="F51" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="17">
+      <c r="F51" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="28">
         <v>50</v>
       </c>
-      <c r="B52" s="31"/>
-      <c r="C52" s="17">
-        <v>3</v>
-      </c>
-      <c r="D52" s="21" t="s">
+      <c r="B52" s="33"/>
+      <c r="C52" s="28">
+        <v>3</v>
+      </c>
+      <c r="D52" s="28" t="s">
         <v>111</v>
       </c>
-      <c r="E52" s="22">
+      <c r="E52" s="30">
         <v>31653</v>
       </c>
-      <c r="F52" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="17">
+      <c r="F52" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="28">
         <v>51</v>
       </c>
-      <c r="B53" s="31"/>
-      <c r="C53" s="17">
-        <v>4</v>
-      </c>
-      <c r="D53" s="21" t="s">
+      <c r="B53" s="33"/>
+      <c r="C53" s="28">
+        <v>4</v>
+      </c>
+      <c r="D53" s="28" t="s">
         <v>106</v>
       </c>
-      <c r="E53" s="10">
+      <c r="E53" s="30">
         <v>37883</v>
       </c>
-      <c r="F53" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="17">
+      <c r="F53" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="28">
         <v>52</v>
       </c>
-      <c r="B54" s="31"/>
-      <c r="C54" s="17">
+      <c r="B54" s="33"/>
+      <c r="C54" s="28">
         <v>5</v>
       </c>
-      <c r="D54" s="21" t="s">
+      <c r="D54" s="28" t="s">
         <v>113</v>
       </c>
-      <c r="E54" s="22">
+      <c r="E54" s="30">
         <v>32743</v>
       </c>
-      <c r="F54" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="17">
+      <c r="F54" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="28">
         <v>53</v>
       </c>
-      <c r="B55" s="31"/>
-      <c r="C55" s="17">
+      <c r="B55" s="33"/>
+      <c r="C55" s="28">
         <v>6</v>
       </c>
-      <c r="D55" s="21" t="s">
+      <c r="D55" s="28" t="s">
         <v>115</v>
       </c>
-      <c r="E55" s="22">
+      <c r="E55" s="30">
         <v>31080</v>
       </c>
-      <c r="F55" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="17">
+      <c r="F55" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="28">
         <v>54</v>
       </c>
-      <c r="B56" s="31"/>
-      <c r="C56" s="17">
+      <c r="B56" s="33"/>
+      <c r="C56" s="28">
         <v>7</v>
       </c>
-      <c r="D56" s="21" t="s">
+      <c r="D56" s="28" t="s">
         <v>117</v>
       </c>
-      <c r="E56" s="22">
+      <c r="E56" s="30">
         <v>35768</v>
       </c>
-      <c r="F56" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="17">
+      <c r="F56" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="28">
         <v>55</v>
       </c>
-      <c r="B57" s="31"/>
-      <c r="C57" s="17">
+      <c r="B57" s="33"/>
+      <c r="C57" s="28">
         <v>8</v>
       </c>
-      <c r="D57" s="21" t="s">
+      <c r="D57" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="E57" s="22">
+      <c r="E57" s="30">
         <v>37226</v>
       </c>
-      <c r="F57" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="17">
+      <c r="F57" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="28">
         <v>56</v>
       </c>
-      <c r="B58" s="31"/>
-      <c r="C58" s="17">
+      <c r="B58" s="33"/>
+      <c r="C58" s="28">
         <v>9</v>
       </c>
-      <c r="D58" s="21" t="s">
+      <c r="D58" s="28" t="s">
         <v>121</v>
       </c>
-      <c r="E58" s="22">
+      <c r="E58" s="30">
         <v>33221</v>
       </c>
-      <c r="F58" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="17">
+      <c r="F58" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="28">
         <v>57</v>
       </c>
-      <c r="B59" s="31"/>
-      <c r="C59" s="17">
+      <c r="B59" s="33"/>
+      <c r="C59" s="28">
         <v>10</v>
       </c>
-      <c r="D59" s="21" t="s">
+      <c r="D59" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="E59" s="10">
+      <c r="E59" s="30">
         <v>34141</v>
       </c>
-      <c r="F59" s="23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="17">
+      <c r="F59" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="28">
         <v>58</v>
       </c>
-      <c r="B60" s="32"/>
-      <c r="C60" s="17">
+      <c r="B60" s="34"/>
+      <c r="C60" s="28">
         <v>11</v>
       </c>
-      <c r="D60" s="21" t="s">
+      <c r="D60" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="E60" s="10">
+      <c r="E60" s="30">
         <v>37409</v>
       </c>
-      <c r="F60" s="23" t="s">
+      <c r="F60" s="28" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>